<commit_message>
Implement OpenCV camera capture and preprocessing
</commit_message>
<xml_diff>
--- a/DEXTRA_Project_Tracker.xlsx
+++ b/DEXTRA_Project_Tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Dextra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dextra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20534BB1-AEB7-410B-A970-6AA606332BC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A7C830-0005-4EAC-91ED-E71C0BEDDCBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview Dashboard" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -347,8 +345,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -574,7 +572,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -586,7 +584,7 @@
     <xf numFmtId="0" fontId="8" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -595,10 +593,10 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1070,13 +1068,13 @@
       <c r="E5" s="2"/>
       <c r="F5" s="24">
         <f>'Trello Board &amp; Tasks'!C6</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="25"/>
       <c r="H5" s="3"/>
       <c r="I5" s="28">
         <f>'Trello Board &amp; Tasks'!C7</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J5" s="25"/>
       <c r="K5" s="4"/>
@@ -1225,7 +1223,7 @@
       </c>
       <c r="C6" s="6">
         <f>COUNTIF(G12:G21, TRUE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" s="6"/>
     </row>
@@ -1235,7 +1233,7 @@
       </c>
       <c r="C7" s="7">
         <f>IF(C5&gt;0, C6/C5, 0)</f>
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D7" s="6"/>
     </row>
@@ -1294,7 +1292,7 @@
         <v>35</v>
       </c>
       <c r="G12" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H12" s="11">
         <v>46199</v>

</xml_diff>

<commit_message>
feat: implement scroll-driven landing page with 3D canvas animations and interactive components
</commit_message>
<xml_diff>
--- a/DEXTRA_Project_Tracker.xlsx
+++ b/DEXTRA_Project_Tracker.xlsx
@@ -1,14 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Dextra\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAE322F1-964E-44EA-A812-C438454E1D80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A82A89D-6208-4023-9858-6D2F2F74BA08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,6 +22,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -34,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="106">
   <si>
     <t>DEXTRA MANAGEMENT CONSOLE &amp; PROGRESS DASHBOARD</t>
   </si>
@@ -63,6 +60,9 @@
     <t>Count</t>
   </si>
   <si>
+    <t>Done</t>
+  </si>
+  <si>
     <t>Salman</t>
   </si>
   <si>
@@ -75,15 +75,18 @@
     <t>In Progress</t>
   </si>
   <si>
+    <t>Godfrey</t>
+  </si>
+  <si>
+    <t>T10</t>
+  </si>
+  <si>
+    <t>2hrs</t>
+  </si>
+  <si>
     <t>Muthamil</t>
   </si>
   <si>
-    <t>Done</t>
-  </si>
-  <si>
-    <t>Godfrey</t>
-  </si>
-  <si>
     <t>DEXTRA PROJECT TASK ALLOTMENT BOARD</t>
   </si>
   <si>
@@ -261,12 +264,12 @@
     <t>Build dark themed sliders/toggles to configure thresholds, camera indices, and custom wakewords.</t>
   </si>
   <si>
+    <t>Frontend/</t>
+  </si>
+  <si>
     <t>Verify Vite local dev server runs on port 5173; verify forms state bindings to FastAPI REST schema.</t>
   </si>
   <si>
-    <t>T10</t>
-  </si>
-  <si>
     <t>Gesture Trainer Console</t>
   </si>
   <si>
@@ -300,6 +303,15 @@
     <t>L01</t>
   </si>
   <si>
+    <t>L02</t>
+  </si>
+  <si>
+    <t>Completed the gui light themed sliders/toggles to configure thresholds, camera indices, and custom wakewords.</t>
+  </si>
+  <si>
+    <t>3hrs</t>
+  </si>
+  <si>
     <t>DEXTRA QA BUG TRACKER &amp; TICKETS</t>
   </si>
   <si>
@@ -336,16 +348,7 @@
     <t>Closed</t>
   </si>
   <si>
-    <t>L02</t>
-  </si>
-  <si>
-    <t>Completed the gui light themed sliders/toggles to configure thresholds, camera indices, and custom wakewords.</t>
-  </si>
-  <si>
-    <t>3hrs</t>
-  </si>
-  <si>
-    <t>Frontend/</t>
+    <t>Developed the UI only..afeter building full backend ..i shall intergrate it..</t>
   </si>
 </sst>
 </file>
@@ -357,7 +360,7 @@
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -378,15 +381,15 @@
       <name val="Segoe UI"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <b/>
       <sz val="20"/>
       <color rgb="FF0F172A"/>
       <name val="Segoe UI"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -410,12 +413,6 @@
       <sz val="10"/>
       <color rgb="FF334155"/>
       <name val="Segoe UI"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="11">
@@ -575,7 +572,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -618,21 +615,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -650,7 +647,7 @@
       </fill>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -679,48 +676,31 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E4279D10-D5D4-3E2A-4344-70CDE3B4C62D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
         <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+          <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="742950" y="2171700"/>
-          <a:ext cx="9198110" cy="5257800"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1013,8 +993,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:S8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B2:S21"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="2" customWidth="1"/>
     <col min="3" max="4" width="14" customWidth="1"/>
@@ -1027,7 +1007,7 @@
     <col min="12" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:19" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="20" t="s">
         <v>0</v>
       </c>
@@ -1039,27 +1019,27 @@
       <c r="H2" s="21"/>
       <c r="I2" s="21"/>
     </row>
-    <row r="4" spans="2:19" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="25"/>
+      <c r="D4" s="23"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="24" t="s">
+      <c r="F4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="25"/>
+      <c r="G4" s="23"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="24" t="s">
+      <c r="I4" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="25"/>
+      <c r="J4" s="23"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="24" t="s">
+      <c r="L4" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="25"/>
+      <c r="M4" s="23"/>
       <c r="O4" s="5" t="s">
         <v>5</v>
       </c>
@@ -1075,38 +1055,37 @@
     </row>
     <row r="5" spans="2:19" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
-      <c r="C5" s="26">
+      <c r="C5" s="24">
         <f>'Trello Board &amp; Tasks'!C5</f>
         <v>10</v>
       </c>
-      <c r="D5" s="27"/>
+      <c r="D5" s="25"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="26">
-        <f>'Trello Board &amp; Tasks'!C6</f>
-        <v>3</v>
-      </c>
-      <c r="G5" s="27"/>
+      <c r="F5" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="25"/>
       <c r="H5" s="3"/>
-      <c r="I5" s="30">
+      <c r="I5" s="28">
         <f>'Trello Board &amp; Tasks'!C7</f>
         <v>0.3</v>
       </c>
-      <c r="J5" s="27"/>
+      <c r="J5" s="25"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="26">
+      <c r="L5" s="24">
         <f>COUNTIF('Bug Tracker &amp; QA Logs'!F$5:F$15, "Open")</f>
         <v>0</v>
       </c>
-      <c r="M5" s="27"/>
+      <c r="M5" s="25"/>
       <c r="O5" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P5" s="5">
         <f>SUMIFS('Trello Board &amp; Tasks'!J$12:J$21, 'Trello Board &amp; Tasks'!C$12:C$21, "Salman")</f>
         <v>5</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="S5" s="5">
         <f>COUNTIF('Trello Board &amp; Tasks'!B$12:B$21, "To Do")</f>
@@ -1115,68 +1094,82 @@
     </row>
     <row r="6" spans="2:19" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="29"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="27"/>
       <c r="E6" s="2"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="29"/>
+      <c r="F6" s="26"/>
+      <c r="G6" s="27"/>
       <c r="H6" s="3"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="29"/>
+      <c r="I6" s="26"/>
+      <c r="J6" s="27"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="28"/>
-      <c r="M6" s="29"/>
+      <c r="L6" s="26"/>
+      <c r="M6" s="27"/>
       <c r="O6" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="P6" s="5">
         <f>SUMIFS('Trello Board &amp; Tasks'!J$12:J$21, 'Trello Board &amp; Tasks'!C$12:C$21, "Logesh")</f>
         <v>5</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="S6" s="5">
         <f>COUNTIF('Trello Board &amp; Tasks'!B$12:B$21, "In Progress")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="2:19" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
+        <v>16</v>
+      </c>
       <c r="O7" s="5" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="P7" s="5">
         <f>SUMIFS('Trello Board &amp; Tasks'!J$12:J$21, 'Trello Board &amp; Tasks'!C$12:C$21, "Muthamil")</f>
         <v>2</v>
       </c>
       <c r="R7" s="5" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="S7" s="5">
         <f>COUNTIF('Trello Board &amp; Tasks'!B$12:B$21, "Done")</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="2:19" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
       <c r="O8" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="P8" s="5">
         <f>SUMIFS('Trello Board &amp; Tasks'!J$12:J$21, 'Trello Board &amp; Tasks'!C$12:C$21, "Godfrey")</f>
         <v>2</v>
       </c>
     </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="C5:D6"/>
+    <mergeCell ref="F5:G6"/>
+    <mergeCell ref="I5:J6"/>
+    <mergeCell ref="L5:M6"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="C4:D4"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="L4:M4"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="F5:G6"/>
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="I5:J6"/>
-    <mergeCell ref="L5:M6"/>
-    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -1186,9 +1179,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:K21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
@@ -1200,9 +1192,9 @@
     <col min="11" max="11" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" s="21"/>
       <c r="C2" s="21"/>
@@ -1215,16 +1207,16 @@
       <c r="J2" s="21"/>
       <c r="K2" s="21"/>
     </row>
-    <row r="4" spans="1:11" ht="16.8" x14ac:dyDescent="0.4">
-      <c r="B4" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-    </row>
-    <row r="5" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="16.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+    </row>
+    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C5" s="6">
         <f>COUNTA(A12:A21)</f>
@@ -1232,9 +1224,9 @@
       </c>
       <c r="D5" s="6"/>
     </row>
-    <row r="6" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C6" s="6">
         <f>COUNTIF(G12:G21, TRUE)</f>
@@ -1242,9 +1234,9 @@
       </c>
       <c r="D6" s="6"/>
     </row>
-    <row r="7" spans="1:11" ht="15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C7" s="7">
         <f>IF(C5&gt;0, C6/C5, 0)</f>
@@ -1252,59 +1244,59 @@
       </c>
       <c r="D7" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G12" s="9" t="b">
         <v>1</v>
@@ -1320,27 +1312,27 @@
         <v>1</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B13" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="13" t="s">
-        <v>9</v>
-      </c>
       <c r="D13" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G13" s="13" t="b">
         <v>0</v>
@@ -1356,27 +1348,27 @@
         <v>2</v>
       </c>
       <c r="K13" s="14" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B14" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="9" t="s">
-        <v>9</v>
-      </c>
       <c r="D14" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G14" s="9" t="b">
         <v>0</v>
@@ -1392,27 +1384,27 @@
         <v>2</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G15" s="13" t="b">
         <v>0</v>
@@ -1428,27 +1420,27 @@
         <v>2</v>
       </c>
       <c r="K15" s="14" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G16" s="9" t="b">
         <v>0</v>
@@ -1464,27 +1456,27 @@
         <v>2</v>
       </c>
       <c r="K16" s="10" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G17" s="13" t="b">
         <v>0</v>
@@ -1500,27 +1492,27 @@
         <v>1</v>
       </c>
       <c r="K17" s="14" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G18" s="9" t="b">
         <v>0</v>
@@ -1536,27 +1528,27 @@
         <v>1</v>
       </c>
       <c r="K18" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G19" s="13" t="b">
         <v>0</v>
@@ -1572,27 +1564,27 @@
         <v>1</v>
       </c>
       <c r="K19" s="14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B20" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="9" t="s">
-        <v>15</v>
-      </c>
       <c r="D20" s="10" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="G20" s="9" t="b">
         <v>1</v>
@@ -1608,27 +1600,27 @@
         <v>1</v>
       </c>
       <c r="K20" s="10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="13" t="s">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D21" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="F21" s="10" t="s">
         <v>77</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="F21" s="10" t="s">
-        <v>103</v>
       </c>
       <c r="G21" s="9" t="b">
         <v>1</v>
@@ -1644,7 +1636,7 @@
         <v>1</v>
       </c>
       <c r="K21" s="14" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1664,7 +1656,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:G10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="3" width="14" customWidth="1"/>
@@ -1674,9 +1666,9 @@
     <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B2" s="21"/>
       <c r="C2" s="21"/>
@@ -1685,86 +1677,98 @@
       <c r="F2" s="21"/>
       <c r="G2" s="21"/>
     </row>
-    <row r="4" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B5" s="11">
         <v>46199</v>
       </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="18"/>
       <c r="G5" s="9"/>
     </row>
-    <row r="6" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B6" s="11">
-        <v>46200</v>
+        <v>46206</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>102</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>14</v>
+        <v>92</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="9"/>
-    </row>
-    <row r="8" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="11">
+        <v>46207</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
       <c r="B8" s="15"/>
       <c r="C8" s="13"/>
       <c r="D8" s="13"/>
       <c r="E8" s="14"/>
       <c r="F8" s="19"/>
-      <c r="G8" s="13"/>
-    </row>
-    <row r="9" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G8" s="9"/>
+    </row>
+    <row r="9" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9"/>
       <c r="B9" s="11"/>
       <c r="C9" s="9"/>
@@ -1773,28 +1777,27 @@
       <c r="F9" s="18"/>
       <c r="G9" s="9"/>
     </row>
-    <row r="10" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13"/>
       <c r="B10" s="15"/>
       <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="14"/>
       <c r="F10" s="19"/>
-      <c r="G10" s="13"/>
+      <c r="G10" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <phoneticPr fontId="9" type="noConversion"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="C5:C10" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Salman,Logesh,Muthamil,Godfrey"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D5:D10" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D5:D10" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"T01,T02,T03,T04,T05,T06,T07,T08,T09,T10"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5" xr:uid="{A09B565B-9577-4881-9939-CD2403D20868}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:G10" xr:uid="{00000000-0002-0000-0200-000004000000}">
       <formula1>"In Progess, Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1805,7 +1808,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A2:I11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -1816,9 +1819,9 @@
     <col min="9" max="9" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B2" s="21"/>
       <c r="C2" s="21"/>
@@ -1829,47 +1832,47 @@
       <c r="H2" s="21"/>
       <c r="I2" s="21"/>
     </row>
-    <row r="4" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="9" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D5" s="10"/>
       <c r="E5" s="9"/>
       <c r="F5" s="9" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="G5" s="11">
         <v>46201</v>
@@ -1879,7 +1882,7 @@
       </c>
       <c r="I5" s="10"/>
     </row>
-    <row r="6" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="13"/>
       <c r="B6" s="14"/>
       <c r="C6" s="13"/>
@@ -1890,11 +1893,11 @@
       <c r="H6" s="15"/>
       <c r="I6" s="14"/>
     </row>
-    <row r="7" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="9" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -1908,7 +1911,7 @@
     <dataValidation type="list" allowBlank="1" sqref="C5:C10" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F5:F10" xr:uid="{00000000-0002-0000-0300-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F5:F10" xr:uid="{00000000-0002-0000-0300-000002000000}">
       <formula1>"Open,Investigation,Resolved,Closed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: add DEXTRA interactive showcase HTML and update project tracker documentation
</commit_message>
<xml_diff>
--- a/DEXTRA_Project_Tracker.xlsx
+++ b/DEXTRA_Project_Tracker.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A82A89D-6208-4023-9858-6D2F2F74BA08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\PROJECTS\Dextra\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{560E78D8-7E68-44F0-B0DB-91870D4973D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-118" yWindow="-118" windowWidth="25370" windowHeight="15945" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview Dashboard" sheetId="1" r:id="rId1"/>
@@ -31,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="153">
   <si>
     <t>DEXTRA MANAGEMENT CONSOLE &amp; PROGRESS DASHBOARD</t>
   </si>
@@ -60,33 +65,30 @@
     <t>Count</t>
   </si>
   <si>
+    <t>Salman</t>
+  </si>
+  <si>
+    <t>To Do</t>
+  </si>
+  <si>
+    <t>Logesh</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Godfrey</t>
+  </si>
+  <si>
+    <t>T10</t>
+  </si>
+  <si>
+    <t>Muthamil</t>
+  </si>
+  <si>
     <t>Done</t>
   </si>
   <si>
-    <t>Salman</t>
-  </si>
-  <si>
-    <t>To Do</t>
-  </si>
-  <si>
-    <t>Logesh</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>Godfrey</t>
-  </si>
-  <si>
-    <t>T10</t>
-  </si>
-  <si>
-    <t>2hrs</t>
-  </si>
-  <si>
-    <t>Muthamil</t>
-  </si>
-  <si>
     <t>DEXTRA PROJECT TASK ALLOTMENT BOARD</t>
   </si>
   <si>
@@ -303,15 +305,99 @@
     <t>L01</t>
   </si>
   <si>
+    <t>Initialized camera capture stream using OpenCV; implemented frame cropping, mirroring, and scaling.</t>
+  </si>
+  <si>
+    <t>4hrs</t>
+  </si>
+  <si>
     <t>L02</t>
   </si>
   <si>
-    <t>Completed the gui light themed sliders/toggles to configure thresholds, camera indices, and custom wakewords.</t>
+    <t>Built thread-safe Config Manager persisting settings and custom gestures to JSON storage.</t>
   </si>
   <si>
     <t>3hrs</t>
   </si>
   <si>
+    <t>L03</t>
+  </si>
+  <si>
+    <t>Built React Settings GUI console with real-time controls for thresholds, camera indices, and wakewords.</t>
+  </si>
+  <si>
+    <t>L04</t>
+  </si>
+  <si>
+    <t>Implemented MediaPipe Hands model landmark tracker extracting 21 3D normalized coordinates.</t>
+  </si>
+  <si>
+    <t>5hrs</t>
+  </si>
+  <si>
+    <t>L05</t>
+  </si>
+  <si>
+    <t>Created mouse execution mapper with NumPy coordinate smoothing and PyAutoGUI click/scroll actions.</t>
+  </si>
+  <si>
+    <t>L06</t>
+  </si>
+  <si>
+    <t>Configured sounddevice background sound recording and ambient noise calibrated wakeword engine.</t>
+  </si>
+  <si>
+    <t>L07</t>
+  </si>
+  <si>
+    <t>Integrated Hugging Face Whisper-tiny transformer pipeline STT speech-to-text decoder.</t>
+  </si>
+  <si>
+    <t>6hrs</t>
+  </si>
+  <si>
+    <t>L08</t>
+  </si>
+  <si>
+    <t>Refined UI dark-themed design system, slider components, and REST API state bindings.</t>
+  </si>
+  <si>
+    <t>L09</t>
+  </si>
+  <si>
+    <t>Developed Gesture Trainer UI canvas with live WebSocket streaming &amp; custom gesture coordinate capture.</t>
+  </si>
+  <si>
+    <t>L10</t>
+  </si>
+  <si>
+    <t>Mapped transcribed voice command keywords to PyAutoGUI OS hotkeys.</t>
+  </si>
+  <si>
+    <t>L11</t>
+  </si>
+  <si>
+    <t>Built FastAPI REST backend &amp; WebSocket endpoints streaming annotated JPEG frames and trainer data.</t>
+  </si>
+  <si>
+    <t>L12</t>
+  </si>
+  <si>
+    <t>T08/B02</t>
+  </si>
+  <si>
+    <t>Diagnosed and fixed WebSocket stream disconnect handling on /trainer/stream &amp; /voice/stream endpoints.</t>
+  </si>
+  <si>
+    <t>L13</t>
+  </si>
+  <si>
+    <t>T02/B03</t>
+  </si>
+  <si>
+    <t>Resolved MediaPipe clearcut telemetry upload connection errors (Status_ConnectFailed: 12029).</t>
+  </si>
+  <si>
     <t>DEXTRA QA BUG TRACKER &amp; TICKETS</t>
   </si>
   <si>
@@ -345,10 +431,70 @@
     <t>Medium</t>
   </si>
   <si>
+    <t>OpenCV VideoCapture camera resource locking on server restart causing frame capture freeze.</t>
+  </si>
+  <si>
     <t>Closed</t>
   </si>
   <si>
-    <t>Developed the UI only..afeter building full backend ..i shall intergrate it..</t>
+    <t>Added try-finally cleanup blocks and explicit camera.release() calls on stream shutdown.</t>
+  </si>
+  <si>
+    <t>B02</t>
+  </si>
+  <si>
+    <t>python/gui_server.py</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>FastAPI WebSocket stream disconnect error on /trainer/stream when client closes connection.</t>
+  </si>
+  <si>
+    <t>Handled WebSocketDisconnect exception gracefully and added client connection manager to prevent crashing worker tasks.</t>
+  </si>
+  <si>
+    <t>B03</t>
+  </si>
+  <si>
+    <t>MediaPipe clearcut telemetry upload failures (Status_ConnectFailed: 12029) due to restricted network.</t>
+  </si>
+  <si>
+    <t>Disabled Clearcut telemetry background uploads via environment configuration and suppressed offline warnings.</t>
+  </si>
+  <si>
+    <t>B04</t>
+  </si>
+  <si>
+    <t>Mouse cursor jitter and accidental double-clicks during fast hand movements.</t>
+  </si>
+  <si>
+    <t>Implemented Exponential Moving Average (EMA) smoothing filter (alpha=0.35) and added click cooldown timer.</t>
+  </si>
+  <si>
+    <t>B05</t>
+  </si>
+  <si>
+    <t>High CPU utilization and audio buffer overflow during continuous background sound recording.</t>
+  </si>
+  <si>
+    <t>Optimized sounddevice blocksize to 1024 samples and implemented ring buffer queue processing.</t>
+  </si>
+  <si>
+    <t>B06</t>
+  </si>
+  <si>
+    <t>Git Repository</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Default tracking branch misalignment and orphan remote tracking branch theoriongd on GitHub.</t>
+  </si>
+  <si>
+    <t>Updated local remote HEAD to dextra branch and deleted obsolete theoriongd branch remotely.</t>
   </si>
 </sst>
 </file>
@@ -477,22 +623,11 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFE2E8F0"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFE2E8F0"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -504,15 +639,6 @@
       <top style="thin">
         <color rgb="FFE2E8F0"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFE2E8F0"/>
-      </left>
-      <right/>
-      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -562,74 +688,125 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="8" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="6" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="6" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -701,6 +878,9 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1007,39 +1187,39 @@
     <col min="12" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:19" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="20" t="s">
+    <row r="2" spans="2:19" ht="42.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-    </row>
-    <row r="4" spans="2:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+    </row>
+    <row r="4" spans="2:19" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1"/>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="23"/>
+      <c r="D4" s="21"/>
       <c r="E4" s="2"/>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="G4" s="23"/>
+      <c r="G4" s="21"/>
       <c r="H4" s="3"/>
-      <c r="I4" s="22" t="s">
+      <c r="I4" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="23"/>
+      <c r="J4" s="21"/>
       <c r="K4" s="4"/>
-      <c r="L4" s="22" t="s">
+      <c r="L4" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="23"/>
+      <c r="M4" s="21"/>
       <c r="O4" s="5" t="s">
         <v>5</v>
       </c>
@@ -1061,14 +1241,15 @@
       </c>
       <c r="D5" s="25"/>
       <c r="E5" s="2"/>
-      <c r="F5" s="24" t="s">
-        <v>9</v>
+      <c r="F5" s="24">
+        <f>'Trello Board &amp; Tasks'!C6</f>
+        <v>10</v>
       </c>
       <c r="G5" s="25"/>
       <c r="H5" s="3"/>
       <c r="I5" s="28">
         <f>'Trello Board &amp; Tasks'!C7</f>
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="J5" s="25"/>
       <c r="K5" s="4"/>
@@ -1078,18 +1259,18 @@
       </c>
       <c r="M5" s="25"/>
       <c r="O5" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P5" s="5">
         <f>SUMIFS('Trello Board &amp; Tasks'!J$12:J$21, 'Trello Board &amp; Tasks'!C$12:C$21, "Salman")</f>
         <v>5</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="S5" s="5">
         <f>COUNTIF('Trello Board &amp; Tasks'!B$12:B$21, "To Do")</f>
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="2:19" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -1106,70 +1287,61 @@
       <c r="L6" s="26"/>
       <c r="M6" s="27"/>
       <c r="O6" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="P6" s="5">
         <f>SUMIFS('Trello Board &amp; Tasks'!J$12:J$21, 'Trello Board &amp; Tasks'!C$12:C$21, "Logesh")</f>
         <v>5</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="S6" s="5">
         <f>COUNTIF('Trello Board &amp; Tasks'!B$12:B$21, "In Progress")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:19" x14ac:dyDescent="0.25">
-      <c r="C7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" t="s">
+    <row r="7" spans="2:19" ht="15.05" x14ac:dyDescent="0.3">
+      <c r="O7" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="F7" t="s">
-        <v>16</v>
-      </c>
-      <c r="O7" s="5" t="s">
-        <v>17</v>
       </c>
       <c r="P7" s="5">
         <f>SUMIFS('Trello Board &amp; Tasks'!J$12:J$21, 'Trello Board &amp; Tasks'!C$12:C$21, "Muthamil")</f>
         <v>2</v>
       </c>
       <c r="R7" s="5" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="S7" s="5">
         <f>COUNTIF('Trello Board &amp; Tasks'!B$12:B$21, "Done")</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="2:19" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="2:19" ht="15.05" x14ac:dyDescent="0.3">
       <c r="O8" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P8" s="5">
         <f>SUMIFS('Trello Board &amp; Tasks'!J$12:J$21, 'Trello Board &amp; Tasks'!C$12:C$21, "Godfrey")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:2" ht="15.05" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="F5:G6"/>
-    <mergeCell ref="I5:J6"/>
-    <mergeCell ref="L5:M6"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="C4:D4"/>
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="L4:M4"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="F5:G6"/>
+    <mergeCell ref="C5:D6"/>
+    <mergeCell ref="I5:J6"/>
+    <mergeCell ref="L5:M6"/>
+    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -1192,31 +1364,31 @@
     <col min="11" max="11" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+    <row r="2" spans="1:11" ht="40.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+    </row>
+    <row r="4" spans="1:11" ht="16.850000000000001" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-    </row>
-    <row r="4" spans="1:11" ht="16.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="29" t="s">
+      <c r="C4" s="30"/>
+      <c r="D4" s="31"/>
+    </row>
+    <row r="5" spans="1:11" ht="15.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="6" t="s">
         <v>19</v>
-      </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-    </row>
-    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="6" t="s">
-        <v>20</v>
       </c>
       <c r="C5" s="6">
         <f>COUNTA(A12:A21)</f>
@@ -1224,79 +1396,79 @@
       </c>
       <c r="D5" s="6"/>
     </row>
-    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="15.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6" s="6">
         <f>COUNTIF(G12:G21, TRUE)</f>
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D6" s="6"/>
     </row>
-    <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="15.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7" s="7">
         <f>IF(C5&gt;0, C6/C5, 0)</f>
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="D7" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="C11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="D11" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="E11" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="F11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="G11" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="H11" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="I11" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="I11" s="8" t="s">
+      <c r="J11" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="K11" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="K11" s="8" t="s">
+    </row>
+    <row r="12" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+      <c r="B12" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="10" t="s">
+      <c r="E12" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="F12" s="10" t="s">
         <v>36</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>37</v>
       </c>
       <c r="G12" s="9" t="b">
         <v>1</v>
@@ -1312,30 +1484,30 @@
         <v>1</v>
       </c>
       <c r="K12" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
+      <c r="B13" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="14" t="s">
+      <c r="E13" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="F13" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="14" t="s">
-        <v>42</v>
-      </c>
       <c r="G13" s="13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H13" s="15">
         <v>46201</v>
@@ -1348,30 +1520,30 @@
         <v>2</v>
       </c>
       <c r="K13" s="14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="B14" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="10" t="s">
+      <c r="E14" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="F14" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>47</v>
-      </c>
       <c r="G14" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" s="11">
         <v>46201</v>
@@ -1384,30 +1556,30 @@
         <v>2</v>
       </c>
       <c r="K14" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="13" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
+      <c r="B15" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="14" t="s">
+      <c r="E15" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="F15" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="F15" s="14" t="s">
-        <v>52</v>
-      </c>
       <c r="G15" s="13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" s="15">
         <v>46204</v>
@@ -1420,30 +1592,30 @@
         <v>2</v>
       </c>
       <c r="K15" s="14" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
+      <c r="B16" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="10" t="s">
+      <c r="E16" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F16" s="10" t="s">
-        <v>57</v>
-      </c>
       <c r="G16" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16" s="11">
         <v>46204</v>
@@ -1456,30 +1628,30 @@
         <v>2</v>
       </c>
       <c r="K16" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="13" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
+      <c r="B17" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="14" t="s">
+      <c r="E17" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="F17" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="F17" s="14" t="s">
-        <v>62</v>
-      </c>
       <c r="G17" s="13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="15">
         <v>46207</v>
@@ -1492,30 +1664,30 @@
         <v>1</v>
       </c>
       <c r="K17" s="14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
+      <c r="B18" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D18" s="10" t="s">
+      <c r="E18" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="F18" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>67</v>
-      </c>
       <c r="G18" s="9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H18" s="11">
         <v>46199</v>
@@ -1528,30 +1700,30 @@
         <v>1</v>
       </c>
       <c r="K18" s="10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="13" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="13" t="s">
+      <c r="B19" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="B19" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="D19" s="14" t="s">
+      <c r="E19" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="E19" s="14" t="s">
+      <c r="F19" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="F19" s="14" t="s">
-        <v>72</v>
-      </c>
       <c r="G19" s="13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="15">
         <v>46207</v>
@@ -1564,27 +1736,27 @@
         <v>1</v>
       </c>
       <c r="K19" s="14" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="9" t="s">
+      <c r="B20" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D20" s="10" t="s">
+      <c r="E20" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="F20" s="10" t="s">
         <v>76</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>77</v>
       </c>
       <c r="G20" s="9" t="b">
         <v>1</v>
@@ -1600,27 +1772,27 @@
         <v>1</v>
       </c>
       <c r="K20" s="10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="60.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="14" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="60.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" s="14" t="s">
+      <c r="E21" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="E21" s="14" t="s">
-        <v>80</v>
-      </c>
       <c r="F21" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G21" s="9" t="b">
         <v>1</v>
@@ -1636,7 +1808,7 @@
         <v>1</v>
       </c>
       <c r="K21" s="14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1655,7 +1827,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A2:G10"/>
+  <dimension ref="A2:G17"/>
   <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1666,125 +1838,338 @@
     <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+    <row r="2" spans="1:7" ht="40.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+    </row>
+    <row r="4" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-    </row>
-    <row r="4" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="B4" s="17" t="s">
         <v>83</v>
-      </c>
-      <c r="B4" s="17" t="s">
-        <v>84</v>
       </c>
       <c r="C4" s="17" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="F4" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="G4" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="G4" s="17" t="s">
+    </row>
+    <row r="5" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>89</v>
       </c>
       <c r="B5" s="11">
         <v>46199</v>
       </c>
-      <c r="C5" s="9"/>
+      <c r="C5" s="9" t="s">
+        <v>9</v>
+      </c>
       <c r="D5" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="9"/>
-    </row>
-    <row r="6" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="11">
+        <v>46199</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="11">
+        <v>46200</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="F7" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="11">
+      <c r="G7" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="11">
+        <v>46201</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="11">
+        <v>46202</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B10" s="11">
+        <v>46204</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" s="11">
+        <v>46205</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F11" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" s="11">
         <v>46206</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C12" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>93</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B13" s="11">
+        <v>46207</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>91</v>
-      </c>
-      <c r="F6" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="G6" s="9" t="s">
+      <c r="E13" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="F13" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15.05" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" s="11">
+        <v>46207</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B15" s="11">
+        <v>46208</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B16" s="11">
+        <v>46226</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B17" s="11">
+        <v>46226</v>
+      </c>
+      <c r="C17" s="9" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="9"/>
-      <c r="B7" s="11">
-        <v>46207</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>92</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="19"/>
-      <c r="G8" s="9"/>
-    </row>
-    <row r="9" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="9"/>
-    </row>
-    <row r="10" spans="1:7" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="9"/>
+      <c r="D17" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="F17" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1794,10 +2179,10 @@
     <dataValidation type="list" allowBlank="1" sqref="C5:C10" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Salman,Logesh,Muthamil,Godfrey"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D5:D10" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D5:D10" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"T01,T02,T03,T04,T05,T06,T07,T08,T09,T10"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:G10" xr:uid="{00000000-0002-0000-0200-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:G10" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"In Progess, Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1819,60 +2204,66 @@
     <col min="9" max="9" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
-        <v>93</v>
-      </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-    </row>
-    <row r="4" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="40.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+    </row>
+    <row r="4" spans="1:9" ht="24.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17" t="s">
-        <v>94</v>
+        <v>121</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>97</v>
+        <v>124</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>98</v>
+        <v>125</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>100</v>
+        <v>127</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="B5" s="10"/>
+        <v>129</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>36</v>
+      </c>
       <c r="C5" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="D5" s="10"/>
-      <c r="E5" s="9"/>
+        <v>130</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>9</v>
+      </c>
       <c r="F5" s="9" t="s">
-        <v>104</v>
+        <v>132</v>
       </c>
       <c r="G5" s="11">
         <v>46201</v>
@@ -1880,24 +2271,156 @@
       <c r="H5" s="11">
         <v>46201</v>
       </c>
-      <c r="I5" s="10"/>
-    </row>
-    <row r="6" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="14"/>
-    </row>
-    <row r="7" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="I5" s="10" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="G6" s="15">
+        <v>46225</v>
+      </c>
+      <c r="H6" s="15">
+        <v>46226</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="G7" s="11">
+        <v>46225</v>
+      </c>
+      <c r="H7" s="11">
+        <v>46226</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="G8" s="15">
+        <v>46205</v>
+      </c>
+      <c r="H8" s="15">
+        <v>46206</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="G9" s="11">
+        <v>46206</v>
+      </c>
+      <c r="H9" s="11">
+        <v>46207</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="G10" s="15">
+        <v>46226</v>
+      </c>
+      <c r="H10" s="15">
+        <v>46226</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="41.4" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
@@ -1911,7 +2434,7 @@
     <dataValidation type="list" allowBlank="1" sqref="C5:C10" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F5:F10" xr:uid="{00000000-0002-0000-0300-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="F5:F10" xr:uid="{00000000-0002-0000-0300-000001000000}">
       <formula1>"Open,Investigation,Resolved,Closed"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>